<commit_message>
Atualizacao dos chamados e do historico
</commit_message>
<xml_diff>
--- a/Solicitacoes.xlsx
+++ b/Solicitacoes.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="281">
   <si>
     <t>Protocolo</t>
   </si>
@@ -579,234 +579,234 @@
     <t>Acesso e busca na rede credenciada</t>
   </si>
   <si>
+    <t>COMPESAPREV_Solicito atualização do Portal para release 2.2.22 para HOMOLOGAÇÃO</t>
+  </si>
+  <si>
+    <t>COMPESAPREV_Solicito atualização do Portal para release 2.2.22 para PRODUÇÃO</t>
+  </si>
+  <si>
+    <t>Compesaprev-Lean- Erro na inclusão de procedimento- OPME</t>
+  </si>
+  <si>
+    <t>Liberação de Relatório Geral de Execução e Biometria / Correção de Bloqueios</t>
+  </si>
+  <si>
+    <t>CompesaPrev - criar usuario WTS para Niecia</t>
+  </si>
+  <si>
+    <t>Acesso rede credenciada com perfil de DEPENDENTE não traz resultados.</t>
+  </si>
+  <si>
+    <t>Os detalhes da CARTEIRINHA não está aparecendo para alguns beneficiários</t>
+  </si>
+  <si>
+    <t>Pendente</t>
+  </si>
+  <si>
+    <t>Não consigo vizualizar o que estão pedindo para ALTERAR quando solicitam alteração cadastral de E-MAIL</t>
+  </si>
+  <si>
+    <t>COMPESPREV - Arquivo retorno com erro na importação</t>
+  </si>
+  <si>
+    <t>COMPESAPREV.NIECIA</t>
+  </si>
+  <si>
+    <t>Processamento de Contas</t>
+  </si>
+  <si>
+    <t>COMPESAPREV - SISTEMA NÃO ESTÁ CONSIDERANDO LIMITADOR PF PARA REEMBOLSO</t>
+  </si>
+  <si>
+    <t>Compesaprev- Lean- Erro log integração</t>
+  </si>
+  <si>
+    <t>Julia Albertim</t>
+  </si>
+  <si>
+    <t>Históricos Atendimentos</t>
+  </si>
+  <si>
+    <t>Não está sendo possível SOLUCIONAR DEMANDAS</t>
+  </si>
+  <si>
+    <t>COMPESAPREV_Painel de sincronização - PLANOS</t>
+  </si>
+  <si>
+    <t>Compesaprev - Complemento II SMS 2531696 – Regra para cálculo de coparticipação</t>
+  </si>
+  <si>
+    <t>Retorno de análise</t>
+  </si>
+  <si>
+    <t>Específico</t>
+  </si>
+  <si>
+    <t>CompesaPrev – Erro na Emissão de Boleto</t>
+  </si>
+  <si>
+    <t>COMPESAPREV- LEAN- RELATORIO- Regulações Vencidas</t>
+  </si>
+  <si>
+    <t>Atualização do AG em Produção - Release 3.65.19 (Ambiente e WTS)</t>
+  </si>
+  <si>
+    <t>Impossibilidade de Auditoria Geral de Biometria na Execução de Eventos (Exigência de Filtro por Prestador)</t>
+  </si>
+  <si>
+    <t>COMPESAPREV – AG: Duplicidade dos eventos solicitados no e-mail do Beneficiario</t>
+  </si>
+  <si>
+    <t>Niécia Morais</t>
+  </si>
+  <si>
+    <t>EVIDENCIAS DO PROBLEMA NO RELATORIO DE PREVIA DE PAGAMENTO</t>
+  </si>
+  <si>
+    <t>Erro na de geração do “Nosso Número” no boleto</t>
+  </si>
+  <si>
+    <t>Alinhamento sobre parametrização de críticas/motivos de negação automáticos (AG / Conecta)</t>
+  </si>
+  <si>
+    <t>Inconsistência no cálculo do prazo em horas úteis</t>
+  </si>
+  <si>
+    <t>Ajuste de permissões e perfis de acesso no AG - Papel de Desenvolvedor aplicado a todos os usuários</t>
+  </si>
+  <si>
+    <t>Falha na integração entre AG Web e Central de Atendimento</t>
+  </si>
+  <si>
+    <t>Compesaprev- Conecta- Erro na autorização</t>
+  </si>
+  <si>
+    <t>Erro ao buscar documento/relatório na Consulta de Autorizações (App)</t>
+  </si>
+  <si>
+    <t>Extrato de Utilização com valores de coparticipações sem a limitação de PF e antes do faturamento ser concluído</t>
+  </si>
+  <si>
+    <t>MOBE | Erro no servidor ao tentar logar.</t>
+  </si>
+  <si>
+    <t>Erro de divergência de cadastro entre o AG e o LEAN</t>
+  </si>
+  <si>
+    <t>Lean / AG (Integração e guias travadas)</t>
+  </si>
+  <si>
+    <t>COMPESAPREV- AG- PROD- Agendamento Regulacao travado</t>
+  </si>
+  <si>
+    <t>Portal não envia e-mails, recuperação de senha e processos parados desde 04/09</t>
+  </si>
+  <si>
+    <t>Histórico financeiro sem a informação individual de todos os beneficiários</t>
+  </si>
+  <si>
+    <t>Dúvida sobre o local para salvar/exportar a Guia Executada no Portal do Prestador</t>
+  </si>
+  <si>
+    <t>Erro no faturamento de pagamentos prestadores</t>
+  </si>
+  <si>
+    <t>COMPESAPREV-CONECTA- Eventos negados, com recibo autorizado</t>
+  </si>
+  <si>
+    <t>Correção – CompesaPrev – Erro de Geração do Código de Barras e Linha Digitável</t>
+  </si>
+  <si>
+    <t>Ajuste no tempo de sessão ativa (timeout) do sistema Lean.</t>
+  </si>
+  <si>
+    <t>ALTERAÇÃO NOME PRESTADOR</t>
+  </si>
+  <si>
+    <t>INFORMATIVOS CONECTA - Como vincular imagem</t>
+  </si>
+  <si>
+    <t>Aguardando Revisão de código</t>
+  </si>
+  <si>
+    <t>CONECTA - Erro na execução de guias | pop-up e bloqueio por biometria</t>
+  </si>
+  <si>
+    <t>COMPESAPREV- AG- AGENDAMENTO com erro Módulo de Regulação: Enviar mensagens Lean e Integracao Iris</t>
+  </si>
+  <si>
+    <t>COMPESAPREV- Conecta- Erro na solicitação dos procedimentos.</t>
+  </si>
+  <si>
+    <t>CONECTA - XML não sai do estado de "Em Processamento"</t>
+  </si>
+  <si>
+    <t>Erro 504 Gateway Time-out no AG e na Central de Atendimento</t>
+  </si>
+  <si>
+    <t>LEAN - Mensagens de prestadores não são exibidas no Lean</t>
+  </si>
+  <si>
+    <t>Guia não disponível para execução de eventos por outros prestadores</t>
+  </si>
+  <si>
+    <t>INSTABILIDADE MÓDULOS</t>
+  </si>
+  <si>
+    <t>ROGERIO.ALMEIDA</t>
+  </si>
+  <si>
+    <t>ANS</t>
+  </si>
+  <si>
+    <t>Critica para gerar XML na Rotina Monitoramento TISS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">APP -  Erro no servidor / buscar dados</t>
+  </si>
+  <si>
+    <t>CON - Impossibilidade adiconar corpo clínico</t>
+  </si>
+  <si>
+    <t>AG - Erro ao importar Tabela Genérica (Aguardando Processamento)</t>
+  </si>
+  <si>
+    <t>MICHEL.HERNANDES</t>
+  </si>
+  <si>
+    <t>Remover permissão de administrador no web.config para usuários não autorizados</t>
+  </si>
+  <si>
+    <t>Códigos folhas gerados errados com mudança de módulo.</t>
+  </si>
+  <si>
+    <t>Erro genérico no faturamento 210.PagamentoPrestadores</t>
+  </si>
+  <si>
+    <t>Erro na geração da limitação de cobrança de PF para o grupo Exames e Terapias</t>
+  </si>
+  <si>
+    <t>Aguardando programacao</t>
+  </si>
+  <si>
+    <t>Eventos autorizados automaticamente ficam "Em análise" no Conecta até finalizar a regulação.</t>
+  </si>
+  <si>
+    <t>E-mail para beneficiário sem detalhamento.</t>
+  </si>
+  <si>
+    <t>HOMOLOGAÇÃO - Atualização do ambiente de homologação para a release 3.65.26</t>
+  </si>
+  <si>
+    <t>Calculo da mensalidade sem redistribuição entre o grupo familiar</t>
+  </si>
+  <si>
+    <t>MOBE - Não foi possível carregar a carteirinha</t>
+  </si>
+  <si>
     <t>Retorno de homologacao</t>
   </si>
   <si>
-    <t>COMPESAPREV_Solicito atualização do Portal para release 2.2.22 para HOMOLOGAÇÃO</t>
-  </si>
-  <si>
-    <t>COMPESAPREV_Solicito atualização do Portal para release 2.2.22 para PRODUÇÃO</t>
-  </si>
-  <si>
-    <t>Compesaprev-Lean- Erro na inclusão de procedimento- OPME</t>
-  </si>
-  <si>
-    <t>Liberação de Relatório Geral de Execução e Biometria / Correção de Bloqueios</t>
-  </si>
-  <si>
-    <t>CompesaPrev - criar usuario WTS para Niecia</t>
-  </si>
-  <si>
-    <t>Acesso rede credenciada com perfil de DEPENDENTE não traz resultados.</t>
-  </si>
-  <si>
-    <t>Os detalhes da CARTEIRINHA não está aparecendo para alguns beneficiários</t>
-  </si>
-  <si>
-    <t>Pendente</t>
-  </si>
-  <si>
-    <t>Não consigo vizualizar o que estão pedindo para ALTERAR quando solicitam alteração cadastral de E-MAIL</t>
-  </si>
-  <si>
-    <t>COMPESPREV - Arquivo retorno com erro na importação</t>
-  </si>
-  <si>
-    <t>COMPESAPREV.NIECIA</t>
-  </si>
-  <si>
-    <t>Processamento de Contas</t>
-  </si>
-  <si>
-    <t>COMPESAPREV - SISTEMA NÃO ESTÁ CONSIDERANDO LIMITADOR PF PARA REEMBOLSO</t>
-  </si>
-  <si>
-    <t>Compesaprev- Lean- Erro log integração</t>
-  </si>
-  <si>
-    <t>Julia Albertim</t>
-  </si>
-  <si>
-    <t>Históricos Atendimentos</t>
-  </si>
-  <si>
-    <t>Não está sendo possível SOLUCIONAR DEMANDAS</t>
-  </si>
-  <si>
-    <t>COMPESAPREV_Painel de sincronização - PLANOS</t>
-  </si>
-  <si>
-    <t>Compesaprev - Complemento II SMS 2531696 – Regra para cálculo de coparticipação</t>
-  </si>
-  <si>
-    <t>Retorno de análise</t>
-  </si>
-  <si>
-    <t>Específico</t>
-  </si>
-  <si>
-    <t>CompesaPrev – Erro na Emissão de Boleto</t>
-  </si>
-  <si>
-    <t>COMPESAPREV- LEAN- RELATORIO- Regulações Vencidas</t>
-  </si>
-  <si>
-    <t>Atualização do AG em Produção - Release 3.65.19 (Ambiente e WTS)</t>
-  </si>
-  <si>
-    <t>Impossibilidade de Auditoria Geral de Biometria na Execução de Eventos (Exigência de Filtro por Prestador)</t>
-  </si>
-  <si>
-    <t>COMPESAPREV – AG: Duplicidade dos eventos solicitados no e-mail do Beneficiario</t>
-  </si>
-  <si>
-    <t>Niécia Morais</t>
-  </si>
-  <si>
-    <t>EVIDENCIAS DO PROBLEMA NO RELATORIO DE PREVIA DE PAGAMENTO</t>
-  </si>
-  <si>
-    <t>Erro na de geração do “Nosso Número” no boleto</t>
-  </si>
-  <si>
-    <t>Alinhamento sobre parametrização de críticas/motivos de negação automáticos (AG / Conecta)</t>
-  </si>
-  <si>
-    <t>Inconsistência no cálculo do prazo em horas úteis</t>
-  </si>
-  <si>
-    <t>Ajuste de permissões e perfis de acesso no AG - Papel de Desenvolvedor aplicado a todos os usuários</t>
-  </si>
-  <si>
-    <t>Falha na integração entre AG Web e Central de Atendimento</t>
-  </si>
-  <si>
-    <t>Compesaprev- Conecta- Erro na autorização</t>
-  </si>
-  <si>
-    <t>Erro ao buscar documento/relatório na Consulta de Autorizações (App)</t>
-  </si>
-  <si>
-    <t>Extrato de Utilização com valores de coparticipações sem a limitação de PF e antes do faturamento ser concluído</t>
-  </si>
-  <si>
-    <t>MOBE | Erro no servidor ao tentar logar.</t>
-  </si>
-  <si>
-    <t>Erro de divergência de cadastro entre o AG e o LEAN</t>
-  </si>
-  <si>
-    <t>Lean / AG (Integração e guias travadas)</t>
-  </si>
-  <si>
-    <t>COMPESAPREV- AG- PROD- Agendamento Regulacao travado</t>
-  </si>
-  <si>
-    <t>Portal não envia e-mails, recuperação de senha e processos parados desde 04/09</t>
-  </si>
-  <si>
-    <t>Histórico financeiro sem a informação individual de todos os beneficiários</t>
-  </si>
-  <si>
-    <t>Dúvida sobre o local para salvar/exportar a Guia Executada no Portal do Prestador</t>
-  </si>
-  <si>
-    <t>Erro no faturamento de pagamentos prestadores</t>
-  </si>
-  <si>
-    <t>COMPESAPREV-CONECTA- Eventos negados, com recibo autorizado</t>
-  </si>
-  <si>
-    <t>Correção – CompesaPrev – Erro de Geração do Código de Barras e Linha Digitável</t>
-  </si>
-  <si>
-    <t>Ajuste no tempo de sessão ativa (timeout) do sistema Lean.</t>
-  </si>
-  <si>
-    <t>ALTERAÇÃO NOME PRESTADOR</t>
-  </si>
-  <si>
-    <t>INFORMATIVOS CONECTA - Como vincular imagem</t>
-  </si>
-  <si>
-    <t>Aguardando Revisão de código</t>
-  </si>
-  <si>
-    <t>CONECTA - Erro na execução de guias | pop-up e bloqueio por biometria</t>
-  </si>
-  <si>
-    <t>COMPESAPREV- AG- AGENDAMENTO com erro Módulo de Regulação: Enviar mensagens Lean e Integracao Iris</t>
-  </si>
-  <si>
-    <t>COMPESAPREV- Conecta- Erro na solicitação dos procedimentos.</t>
-  </si>
-  <si>
-    <t>CONECTA - XML não sai do estado de "Em Processamento"</t>
-  </si>
-  <si>
-    <t>Erro 504 Gateway Time-out no AG e na Central de Atendimento</t>
-  </si>
-  <si>
-    <t>LEAN - Mensagens de prestadores não são exibidas no Lean</t>
-  </si>
-  <si>
-    <t>Guia não disponível para execução de eventos por outros prestadores</t>
-  </si>
-  <si>
-    <t>INSTABILIDADE MÓDULOS</t>
-  </si>
-  <si>
-    <t>ROGERIO.ALMEIDA</t>
-  </si>
-  <si>
-    <t>ANS</t>
-  </si>
-  <si>
-    <t>Critica para gerar XML na Rotina Monitoramento TISS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">APP -  Erro no servidor / buscar dados</t>
-  </si>
-  <si>
-    <t>CON - Impossibilidade adiconar corpo clínico</t>
-  </si>
-  <si>
-    <t>AG - Erro ao importar Tabela Genérica (Aguardando Processamento)</t>
-  </si>
-  <si>
-    <t>MICHEL.HERNANDES</t>
-  </si>
-  <si>
-    <t>Remover permissão de administrador no web.config para usuários não autorizados</t>
-  </si>
-  <si>
-    <t>Códigos folhas gerados errados com mudança de módulo.</t>
-  </si>
-  <si>
-    <t>Erro genérico no faturamento 210.PagamentoPrestadores</t>
-  </si>
-  <si>
-    <t>Erro na geração da limitação de cobrança de PF para o grupo Exames e Terapias</t>
-  </si>
-  <si>
-    <t>Aguardando programacao</t>
-  </si>
-  <si>
-    <t>Eventos autorizados automaticamente ficam "Em análise" no Conecta até finalizar a regulação.</t>
-  </si>
-  <si>
-    <t>E-mail para beneficiário sem detalhamento.</t>
-  </si>
-  <si>
-    <t>HOMOLOGAÇÃO - Atualização do ambiente de homologação para a release 3.65.26</t>
-  </si>
-  <si>
-    <t>Calculo da mensalidade sem redistribuição entre o grupo familiar</t>
-  </si>
-  <si>
-    <t>MOBE - Não foi possível carregar a carteirinha</t>
-  </si>
-  <si>
     <t>MOBE - Beneficiário não consegue logar pelo app há mais de um mês</t>
   </si>
   <si>
@@ -840,7 +840,22 @@
     <t>RELATORIO DE PREVIA NÃO GERADO APÓS REPROCESSAMENTO DE PAGAMENTO</t>
   </si>
   <si>
+    <t>Aguardando detalhamento</t>
+  </si>
+  <si>
     <t>baixa de títulos – Importação do arquivo de retorno da folha está baixando a obrigação errada</t>
+  </si>
+  <si>
+    <t>AG - Tombamento – Origem: Produção / Destino: Homologação</t>
+  </si>
+  <si>
+    <t>PORTAL - Tombamento – Origem: Produção / Destino: Homologação</t>
+  </si>
+  <si>
+    <t>LEAN - Tombamento – Origem: Produção / Destino: Homologação</t>
+  </si>
+  <si>
+    <t>Ocultar códigos de glosa TISS na consulta de autorizações do beneficiário</t>
   </si>
 </sst>
 </file>
@@ -896,7 +911,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O169"/>
+  <dimension ref="A1:O173"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.1506990705218" customWidth="1"/>
@@ -4847,16 +4862,16 @@
         <v>181</v>
       </c>
       <c r="H90" s="0" t="s">
-        <v>114</v>
+        <v>165</v>
       </c>
       <c r="I90" s="3">
-        <v>46290.75</v>
+        <v>46304.7916666667</v>
       </c>
       <c r="J90" s="3">
-        <v>46300.6920023148</v>
+        <v>46304.7643055556</v>
       </c>
       <c r="K90" s="0" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="L90" s="0" t="s">
         <v>22</v>
@@ -5025,16 +5040,16 @@
         <v>187</v>
       </c>
       <c r="H94" s="0" t="s">
-        <v>188</v>
+        <v>165</v>
       </c>
       <c r="I94" s="3">
-        <v>46233.3931597222</v>
+        <v>46304.4505787037</v>
       </c>
       <c r="J94" s="3">
-        <v>46304.4505787037</v>
+        <v>46304.7603240741</v>
       </c>
       <c r="K94" s="0" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="L94" s="0" t="s">
         <v>94</v>
@@ -5067,7 +5082,7 @@
         <v>18</v>
       </c>
       <c r="G95" s="0" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="H95" s="0" t="s">
         <v>20</v>
@@ -5112,7 +5127,7 @@
         <v>18</v>
       </c>
       <c r="G96" s="0" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="H96" s="0" t="s">
         <v>20</v>
@@ -5157,7 +5172,7 @@
         <v>80</v>
       </c>
       <c r="G97" s="0" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="H97" s="0" t="s">
         <v>20</v>
@@ -5202,7 +5217,7 @@
         <v>102</v>
       </c>
       <c r="G98" s="0" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="H98" s="0" t="s">
         <v>21</v>
@@ -5247,7 +5262,7 @@
         <v>26</v>
       </c>
       <c r="G99" s="0" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H99" s="0" t="s">
         <v>20</v>
@@ -5292,7 +5307,7 @@
         <v>46</v>
       </c>
       <c r="G100" s="0" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="H100" s="0" t="s">
         <v>20</v>
@@ -5337,10 +5352,10 @@
         <v>38</v>
       </c>
       <c r="G101" s="0" t="s">
+        <v>194</v>
+      </c>
+      <c r="H101" s="0" t="s">
         <v>195</v>
-      </c>
-      <c r="H101" s="0" t="s">
-        <v>196</v>
       </c>
       <c r="I101" s="3">
         <v>46271.3406597222</v>
@@ -5382,7 +5397,7 @@
         <v>38</v>
       </c>
       <c r="G102" s="0" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="H102" s="0" t="s">
         <v>20</v>
@@ -5427,7 +5442,7 @@
         <v>53</v>
       </c>
       <c r="G103" s="0" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="H103" s="0" t="s">
         <v>20</v>
@@ -5457,7 +5472,7 @@
         <v>2598767</v>
       </c>
       <c r="B104" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C104" s="0" t="s">
         <v>129</v>
@@ -5469,10 +5484,10 @@
         <v>17</v>
       </c>
       <c r="F104" s="0" t="s">
+        <v>199</v>
+      </c>
+      <c r="G104" s="0" t="s">
         <v>200</v>
-      </c>
-      <c r="G104" s="0" t="s">
-        <v>201</v>
       </c>
       <c r="H104" s="0" t="s">
         <v>165</v>
@@ -5517,7 +5532,7 @@
         <v>148</v>
       </c>
       <c r="G105" s="0" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="H105" s="0" t="s">
         <v>43</v>
@@ -5550,7 +5565,7 @@
         <v>184</v>
       </c>
       <c r="C106" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D106" s="0" t="s">
         <v>25</v>
@@ -5559,10 +5574,10 @@
         <v>111</v>
       </c>
       <c r="F106" s="0" t="s">
+        <v>203</v>
+      </c>
+      <c r="G106" s="0" t="s">
         <v>204</v>
-      </c>
-      <c r="G106" s="0" t="s">
-        <v>205</v>
       </c>
       <c r="H106" s="0" t="s">
         <v>20</v>
@@ -5607,7 +5622,7 @@
         <v>18</v>
       </c>
       <c r="G107" s="0" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H107" s="0" t="s">
         <v>20</v>
@@ -5652,17 +5667,17 @@
         <v>53</v>
       </c>
       <c r="G108" s="0" t="s">
+        <v>206</v>
+      </c>
+      <c r="H108" s="0" t="s">
         <v>207</v>
-      </c>
-      <c r="H108" s="0" t="s">
-        <v>208</v>
       </c>
       <c r="I108" s="3"/>
       <c r="J108" s="3">
-        <v>46303.4457064815</v>
+        <v>46308.3571082176</v>
       </c>
       <c r="K108" s="0" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="L108" s="0" t="s">
         <v>36</v>
@@ -5693,7 +5708,7 @@
         <v>38</v>
       </c>
       <c r="G109" s="0" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H109" s="0" t="s">
         <v>123</v>
@@ -5722,7 +5737,7 @@
         <v>184</v>
       </c>
       <c r="C110" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D110" s="0" t="s">
         <v>25</v>
@@ -5779,10 +5794,10 @@
         <v>80</v>
       </c>
       <c r="G111" s="0" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H111" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I111" s="3">
         <v>46259.3446296296</v>
@@ -5812,7 +5827,7 @@
         <v>184</v>
       </c>
       <c r="C112" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D112" s="0" t="s">
         <v>25</v>
@@ -5824,7 +5839,7 @@
         <v>18</v>
       </c>
       <c r="G112" s="0" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H112" s="0" t="s">
         <v>20</v>
@@ -5857,7 +5872,7 @@
         <v>184</v>
       </c>
       <c r="C113" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D113" s="0" t="s">
         <v>25</v>
@@ -5869,7 +5884,7 @@
         <v>102</v>
       </c>
       <c r="G113" s="0" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H113" s="0" t="s">
         <v>165</v>
@@ -5914,10 +5929,10 @@
         <v>38</v>
       </c>
       <c r="G114" s="0" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="H114" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I114" s="3">
         <v>46265.3599537037</v>
@@ -5944,10 +5959,10 @@
         <v>2607198</v>
       </c>
       <c r="B115" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C115" s="0" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D115" s="0" t="s">
         <v>25</v>
@@ -5956,10 +5971,10 @@
         <v>17</v>
       </c>
       <c r="F115" s="0" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G115" s="0" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H115" s="0" t="s">
         <v>20</v>
@@ -6004,7 +6019,7 @@
         <v>53</v>
       </c>
       <c r="G116" s="0" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="H116" s="0" t="s">
         <v>20</v>
@@ -6033,7 +6048,7 @@
         <v>184</v>
       </c>
       <c r="C117" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D117" s="0" t="s">
         <v>25</v>
@@ -6045,7 +6060,7 @@
         <v>18</v>
       </c>
       <c r="G117" s="0" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H117" s="0" t="s">
         <v>20</v>
@@ -6078,7 +6093,7 @@
         <v>184</v>
       </c>
       <c r="C118" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D118" s="0" t="s">
         <v>25</v>
@@ -6090,7 +6105,7 @@
         <v>98</v>
       </c>
       <c r="G118" s="0" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H118" s="0" t="s">
         <v>20</v>
@@ -6123,7 +6138,7 @@
         <v>184</v>
       </c>
       <c r="C119" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D119" s="0" t="s">
         <v>25</v>
@@ -6135,7 +6150,7 @@
         <v>18</v>
       </c>
       <c r="G119" s="0" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="H119" s="0" t="s">
         <v>20</v>
@@ -6180,10 +6195,10 @@
         <v>112</v>
       </c>
       <c r="G120" s="0" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H120" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I120" s="3">
         <v>46273.6887962963</v>
@@ -6225,7 +6240,7 @@
         <v>118</v>
       </c>
       <c r="G121" s="0" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="H121" s="0" t="s">
         <v>21</v>
@@ -6270,10 +6285,10 @@
         <v>46</v>
       </c>
       <c r="G122" s="0" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H122" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I122" s="3">
         <v>46301.4629166667</v>
@@ -6300,10 +6315,10 @@
         <v>2610030</v>
       </c>
       <c r="B123" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C123" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D123" s="0" t="s">
         <v>25</v>
@@ -6315,10 +6330,10 @@
         <v>46</v>
       </c>
       <c r="G123" s="0" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H123" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I123" s="3">
         <v>46269.4396990741</v>
@@ -6360,10 +6375,10 @@
         <v>46</v>
       </c>
       <c r="G124" s="0" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H124" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I124" s="3">
         <v>46304.3672569444</v>
@@ -6390,10 +6405,10 @@
         <v>2611521</v>
       </c>
       <c r="B125" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C125" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D125" s="0" t="s">
         <v>25</v>
@@ -6405,10 +6420,10 @@
         <v>38</v>
       </c>
       <c r="G125" s="0" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H125" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I125" s="3">
         <v>46279.3705439815</v>
@@ -6438,7 +6453,7 @@
         <v>184</v>
       </c>
       <c r="C126" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D126" s="0" t="s">
         <v>25</v>
@@ -6450,7 +6465,7 @@
         <v>148</v>
       </c>
       <c r="G126" s="0" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H126" s="0" t="s">
         <v>20</v>
@@ -6495,7 +6510,7 @@
         <v>137</v>
       </c>
       <c r="G127" s="0" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H127" s="0" t="s">
         <v>20</v>
@@ -6528,7 +6543,7 @@
         <v>184</v>
       </c>
       <c r="C128" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D128" s="0" t="s">
         <v>25</v>
@@ -6540,7 +6555,7 @@
         <v>18</v>
       </c>
       <c r="G128" s="0" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H128" s="0" t="s">
         <v>20</v>
@@ -6570,10 +6585,10 @@
         <v>2611692</v>
       </c>
       <c r="B129" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C129" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D129" s="0" t="s">
         <v>25</v>
@@ -6585,10 +6600,10 @@
         <v>46</v>
       </c>
       <c r="G129" s="0" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="H129" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I129" s="3">
         <v>46274.7471527778</v>
@@ -6618,7 +6633,7 @@
         <v>184</v>
       </c>
       <c r="C130" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D130" s="0" t="s">
         <v>25</v>
@@ -6630,7 +6645,7 @@
         <v>102</v>
       </c>
       <c r="G130" s="0" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H130" s="0" t="s">
         <v>165</v>
@@ -6660,10 +6675,10 @@
         <v>2611881</v>
       </c>
       <c r="B131" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C131" s="0" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D131" s="0" t="s">
         <v>25</v>
@@ -6672,10 +6687,10 @@
         <v>17</v>
       </c>
       <c r="F131" s="0" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G131" s="0" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="H131" s="0" t="s">
         <v>20</v>
@@ -6720,10 +6735,10 @@
         <v>118</v>
       </c>
       <c r="G132" s="0" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="H132" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I132" s="3">
         <v>46316.6011689815</v>
@@ -6765,7 +6780,7 @@
         <v>53</v>
       </c>
       <c r="G133" s="0" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="H133" s="0" t="s">
         <v>20</v>
@@ -6798,7 +6813,7 @@
         <v>184</v>
       </c>
       <c r="C134" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D134" s="0" t="s">
         <v>25</v>
@@ -6810,7 +6825,7 @@
         <v>98</v>
       </c>
       <c r="G134" s="0" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H134" s="0" t="s">
         <v>20</v>
@@ -6843,7 +6858,7 @@
         <v>184</v>
       </c>
       <c r="C135" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D135" s="0" t="s">
         <v>25</v>
@@ -6855,7 +6870,7 @@
         <v>121</v>
       </c>
       <c r="G135" s="0" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H135" s="0" t="s">
         <v>20</v>
@@ -6888,7 +6903,7 @@
         <v>184</v>
       </c>
       <c r="C136" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D136" s="0" t="s">
         <v>151</v>
@@ -6900,10 +6915,10 @@
         <v>102</v>
       </c>
       <c r="G136" s="0" t="s">
+        <v>236</v>
+      </c>
+      <c r="H136" s="0" t="s">
         <v>237</v>
-      </c>
-      <c r="H136" s="0" t="s">
-        <v>238</v>
       </c>
       <c r="I136" s="3">
         <v>46303.7916666667</v>
@@ -6933,7 +6948,7 @@
         <v>184</v>
       </c>
       <c r="C137" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D137" s="0" t="s">
         <v>25</v>
@@ -6945,7 +6960,7 @@
         <v>133</v>
       </c>
       <c r="G137" s="0" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="H137" s="0" t="s">
         <v>21</v>
@@ -6990,10 +7005,10 @@
         <v>137</v>
       </c>
       <c r="G138" s="0" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="H138" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I138" s="3">
         <v>46321.5908449074</v>
@@ -7035,7 +7050,7 @@
         <v>118</v>
       </c>
       <c r="G139" s="0" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="H139" s="0" t="s">
         <v>21</v>
@@ -7068,7 +7083,7 @@
         <v>184</v>
       </c>
       <c r="C140" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D140" s="0" t="s">
         <v>25</v>
@@ -7080,7 +7095,7 @@
         <v>133</v>
       </c>
       <c r="G140" s="0" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="H140" s="0" t="s">
         <v>21</v>
@@ -7113,7 +7128,7 @@
         <v>184</v>
       </c>
       <c r="C141" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D141" s="0" t="s">
         <v>25</v>
@@ -7125,7 +7140,7 @@
         <v>18</v>
       </c>
       <c r="G141" s="0" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H141" s="0" t="s">
         <v>20</v>
@@ -7170,10 +7185,10 @@
         <v>18</v>
       </c>
       <c r="G142" s="0" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="H142" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I142" s="3">
         <v>46290.4043865741</v>
@@ -7203,7 +7218,7 @@
         <v>184</v>
       </c>
       <c r="C143" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D143" s="0" t="s">
         <v>50</v>
@@ -7215,7 +7230,7 @@
         <v>133</v>
       </c>
       <c r="G143" s="0" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="H143" s="0" t="s">
         <v>21</v>
@@ -7244,7 +7259,7 @@
         <v>184</v>
       </c>
       <c r="C144" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D144" s="0" t="s">
         <v>25</v>
@@ -7256,7 +7271,7 @@
         <v>18</v>
       </c>
       <c r="G144" s="0" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="H144" s="0" t="s">
         <v>165</v>
@@ -7286,10 +7301,10 @@
         <v>2617933</v>
       </c>
       <c r="B145" s="0" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C145" s="0" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D145" s="0" t="s">
         <v>151</v>
@@ -7298,10 +7313,10 @@
         <v>17</v>
       </c>
       <c r="F145" s="0" t="s">
+        <v>247</v>
+      </c>
+      <c r="G145" s="0" t="s">
         <v>248</v>
-      </c>
-      <c r="G145" s="0" t="s">
-        <v>249</v>
       </c>
       <c r="H145" s="0" t="s">
         <v>20</v>
@@ -7334,7 +7349,7 @@
         <v>184</v>
       </c>
       <c r="C146" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D146" s="0" t="s">
         <v>25</v>
@@ -7346,19 +7361,19 @@
         <v>46</v>
       </c>
       <c r="G146" s="0" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="H146" s="0" t="s">
-        <v>188</v>
+        <v>165</v>
       </c>
       <c r="I146" s="3">
-        <v>46289.4621296296</v>
+        <v>46304.3689699074</v>
       </c>
       <c r="J146" s="3">
-        <v>46304.3689699074</v>
+        <v>46304.7647685185</v>
       </c>
       <c r="K146" s="0" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="L146" s="0" t="s">
         <v>108</v>
@@ -7379,7 +7394,7 @@
         <v>184</v>
       </c>
       <c r="C147" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D147" s="0" t="s">
         <v>25</v>
@@ -7391,7 +7406,7 @@
         <v>163</v>
       </c>
       <c r="G147" s="0" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="H147" s="0" t="s">
         <v>165</v>
@@ -7424,7 +7439,7 @@
         <v>184</v>
       </c>
       <c r="C148" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D148" s="0" t="s">
         <v>25</v>
@@ -7436,19 +7451,19 @@
         <v>18</v>
       </c>
       <c r="G148" s="0" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="H148" s="0" t="s">
-        <v>165</v>
+        <v>20</v>
       </c>
       <c r="I148" s="3">
         <v>46304.3604861111</v>
       </c>
       <c r="J148" s="3">
-        <v>46304.3793865741</v>
+        <v>46304.6581134259</v>
       </c>
       <c r="K148" s="0" t="s">
-        <v>166</v>
+        <v>21</v>
       </c>
       <c r="L148" s="0" t="s">
         <v>94</v>
@@ -7466,10 +7481,10 @@
         <v>2618956</v>
       </c>
       <c r="B149" s="0" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C149" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D149" s="0" t="s">
         <v>16</v>
@@ -7481,7 +7496,7 @@
         <v>92</v>
       </c>
       <c r="G149" s="0" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="H149" s="0" t="s">
         <v>20</v>
@@ -7509,10 +7524,10 @@
         <v>2619015</v>
       </c>
       <c r="B150" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C150" s="0" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D150" s="0" t="s">
         <v>25</v>
@@ -7524,7 +7539,7 @@
         <v>53</v>
       </c>
       <c r="G150" s="0" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="H150" s="0" t="s">
         <v>165</v>
@@ -7566,10 +7581,10 @@
         <v>17</v>
       </c>
       <c r="F151" s="0" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G151" s="0" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="H151" s="0" t="s">
         <v>20</v>
@@ -7599,10 +7614,10 @@
         <v>2619693</v>
       </c>
       <c r="B152" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C152" s="0" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D152" s="0" t="s">
         <v>151</v>
@@ -7614,10 +7629,10 @@
         <v>53</v>
       </c>
       <c r="G152" s="0" t="s">
+        <v>256</v>
+      </c>
+      <c r="H152" s="0" t="s">
         <v>257</v>
-      </c>
-      <c r="H152" s="0" t="s">
-        <v>258</v>
       </c>
       <c r="I152" s="3">
         <v>46294.4604976852</v>
@@ -7626,7 +7641,7 @@
         <v>46302.786412037</v>
       </c>
       <c r="K152" s="0" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="L152" s="0" t="s">
         <v>94</v>
@@ -7647,7 +7662,7 @@
         <v>184</v>
       </c>
       <c r="C153" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D153" s="0" t="s">
         <v>25</v>
@@ -7659,7 +7674,7 @@
         <v>118</v>
       </c>
       <c r="G153" s="0" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="H153" s="0" t="s">
         <v>165</v>
@@ -7704,10 +7719,10 @@
         <v>41</v>
       </c>
       <c r="G154" s="0" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="H154" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I154" s="3">
         <v>46296.426724537</v>
@@ -7737,7 +7752,7 @@
         <v>184</v>
       </c>
       <c r="C155" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D155" s="0" t="s">
         <v>25</v>
@@ -7749,7 +7764,7 @@
         <v>18</v>
       </c>
       <c r="G155" s="0" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="H155" s="0" t="s">
         <v>20</v>
@@ -7779,10 +7794,10 @@
         <v>2620853</v>
       </c>
       <c r="B156" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C156" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D156" s="0" t="s">
         <v>25</v>
@@ -7794,10 +7809,10 @@
         <v>53</v>
       </c>
       <c r="G156" s="0" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="H156" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I156" s="3">
         <v>46300.6124768518</v>
@@ -7827,7 +7842,7 @@
         <v>184</v>
       </c>
       <c r="C157" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D157" s="0" t="s">
         <v>25</v>
@@ -7839,10 +7854,10 @@
         <v>46</v>
       </c>
       <c r="G157" s="0" t="s">
+        <v>262</v>
+      </c>
+      <c r="H157" s="0" t="s">
         <v>263</v>
-      </c>
-      <c r="H157" s="0" t="s">
-        <v>188</v>
       </c>
       <c r="I157" s="3">
         <v>46296.6557523148</v>
@@ -7872,7 +7887,7 @@
         <v>184</v>
       </c>
       <c r="C158" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D158" s="0" t="s">
         <v>25</v>
@@ -7887,16 +7902,16 @@
         <v>264</v>
       </c>
       <c r="H158" s="0" t="s">
-        <v>188</v>
+        <v>165</v>
       </c>
       <c r="I158" s="3">
         <v>46303.4590972222</v>
       </c>
       <c r="J158" s="3">
-        <v>46303.4631783565</v>
+        <v>46304.6906481481</v>
       </c>
       <c r="K158" s="0" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="L158" s="0" t="s">
         <v>94</v>
@@ -7917,7 +7932,7 @@
         <v>184</v>
       </c>
       <c r="C159" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D159" s="0" t="s">
         <v>25</v>
@@ -7962,7 +7977,7 @@
         <v>184</v>
       </c>
       <c r="C160" s="0" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D160" s="0" t="s">
         <v>25</v>
@@ -8049,10 +8064,10 @@
         <v>2623093</v>
       </c>
       <c r="B162" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C162" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D162" s="0" t="s">
         <v>25</v>
@@ -8061,13 +8076,13 @@
         <v>17</v>
       </c>
       <c r="F162" s="0" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G162" s="0" t="s">
         <v>268</v>
       </c>
       <c r="H162" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I162" s="3">
         <v>46301.5634027778</v>
@@ -8112,7 +8127,7 @@
         <v>269</v>
       </c>
       <c r="H163" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I163" s="3">
         <v>46300.6718634259</v>
@@ -8142,7 +8157,7 @@
         <v>184</v>
       </c>
       <c r="C164" s="0" t="s">
-        <v>184</v>
+        <v>202</v>
       </c>
       <c r="D164" s="0" t="s">
         <v>25</v>
@@ -8157,16 +8172,16 @@
         <v>270</v>
       </c>
       <c r="H164" s="0" t="s">
-        <v>196</v>
+        <v>165</v>
       </c>
       <c r="I164" s="3">
         <v>46316.6666666667</v>
       </c>
       <c r="J164" s="3">
-        <v>46301.9862391204</v>
+        <v>46304.4752430556</v>
       </c>
       <c r="K164" s="0" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="L164" s="0" t="s">
         <v>28</v>
@@ -8184,10 +8199,10 @@
         <v>2623556</v>
       </c>
       <c r="B165" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C165" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D165" s="0" t="s">
         <v>25</v>
@@ -8196,13 +8211,13 @@
         <v>17</v>
       </c>
       <c r="F165" s="0" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G165" s="0" t="s">
         <v>271</v>
       </c>
       <c r="H165" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I165" s="3">
         <v>46303.5816898148</v>
@@ -8247,7 +8262,7 @@
         <v>272</v>
       </c>
       <c r="H166" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I166" s="3">
         <v>46304.4082060185</v>
@@ -8274,10 +8289,10 @@
         <v>2625581</v>
       </c>
       <c r="B167" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C167" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D167" s="0" t="s">
         <v>25</v>
@@ -8292,13 +8307,13 @@
         <v>273</v>
       </c>
       <c r="H167" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I167" s="3">
         <v>46308.4791666667</v>
       </c>
       <c r="J167" s="3">
-        <v>46304.3588671296</v>
+        <v>46308.3884850694</v>
       </c>
       <c r="K167" s="0" t="s">
         <v>159</v>
@@ -8319,10 +8334,10 @@
         <v>2625583</v>
       </c>
       <c r="B168" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C168" s="0" t="s">
-        <v>199</v>
+        <v>214</v>
       </c>
       <c r="D168" s="0" t="s">
         <v>25</v>
@@ -8331,19 +8346,19 @@
         <v>17</v>
       </c>
       <c r="F168" s="0" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G168" s="0" t="s">
         <v>274</v>
       </c>
       <c r="H168" s="0" t="s">
-        <v>196</v>
+        <v>275</v>
       </c>
       <c r="I168" s="3">
         <v>46308.4791666667</v>
       </c>
       <c r="J168" s="3">
-        <v>46304.3585439468</v>
+        <v>46304.7359606481</v>
       </c>
       <c r="K168" s="0" t="s">
         <v>159</v>
@@ -8364,10 +8379,10 @@
         <v>2625588</v>
       </c>
       <c r="B169" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C169" s="0" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D169" s="0" t="s">
         <v>25</v>
@@ -8379,16 +8394,16 @@
         <v>53</v>
       </c>
       <c r="G169" s="0" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="H169" s="0" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I169" s="3">
         <v>46308.4791666667</v>
       </c>
       <c r="J169" s="3">
-        <v>46304.3579076042</v>
+        <v>46308.3195029745</v>
       </c>
       <c r="K169" s="0" t="s">
         <v>159</v>
@@ -8403,6 +8418,186 @@
         <v>46308.4791666667</v>
       </c>
       <c r="O169" s="3"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="2">
+        <v>2626013</v>
+      </c>
+      <c r="B170" s="0" t="s">
+        <v>184</v>
+      </c>
+      <c r="C170" s="0" t="s">
+        <v>184</v>
+      </c>
+      <c r="D170" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="E170" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="F170" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="G170" s="0" t="s">
+        <v>277</v>
+      </c>
+      <c r="H170" s="0" t="s">
+        <v>195</v>
+      </c>
+      <c r="I170" s="3">
+        <v>46310.6272800926</v>
+      </c>
+      <c r="J170" s="3">
+        <v>46304.713774456</v>
+      </c>
+      <c r="K170" s="0" t="s">
+        <v>159</v>
+      </c>
+      <c r="L170" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="M170" s="3">
+        <v>46304.6897800926</v>
+      </c>
+      <c r="N170" s="3">
+        <v>46310.6272800926</v>
+      </c>
+      <c r="O170" s="3"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="2">
+        <v>2626021</v>
+      </c>
+      <c r="B171" s="0" t="s">
+        <v>184</v>
+      </c>
+      <c r="C171" s="0" t="s">
+        <v>184</v>
+      </c>
+      <c r="D171" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="E171" s="0" t="s">
+        <v>76</v>
+      </c>
+      <c r="F171" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="G171" s="0" t="s">
+        <v>278</v>
+      </c>
+      <c r="H171" s="0" t="s">
+        <v>195</v>
+      </c>
+      <c r="I171" s="3">
+        <v>46310.6278703704</v>
+      </c>
+      <c r="J171" s="3">
+        <v>46308.3920169329</v>
+      </c>
+      <c r="K171" s="0" t="s">
+        <v>159</v>
+      </c>
+      <c r="L171" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="M171" s="3">
+        <v>46304.6903703704</v>
+      </c>
+      <c r="N171" s="3">
+        <v>46310.6278703704</v>
+      </c>
+      <c r="O171" s="3"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="2">
+        <v>2626022</v>
+      </c>
+      <c r="B172" s="0" t="s">
+        <v>184</v>
+      </c>
+      <c r="C172" s="0" t="s">
+        <v>184</v>
+      </c>
+      <c r="D172" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="E172" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="F172" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="G172" s="0" t="s">
+        <v>279</v>
+      </c>
+      <c r="H172" s="0" t="s">
+        <v>195</v>
+      </c>
+      <c r="I172" s="3">
+        <v>46310.6288310185</v>
+      </c>
+      <c r="J172" s="3">
+        <v>46308.5364623495</v>
+      </c>
+      <c r="K172" s="0" t="s">
+        <v>159</v>
+      </c>
+      <c r="L172" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="M172" s="3">
+        <v>46304.6913310185</v>
+      </c>
+      <c r="N172" s="3">
+        <v>46310.6288310185</v>
+      </c>
+      <c r="O172" s="3"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="2">
+        <v>2626208</v>
+      </c>
+      <c r="B173" s="0" t="s">
+        <v>184</v>
+      </c>
+      <c r="C173" s="0" t="s">
+        <v>184</v>
+      </c>
+      <c r="D173" s="0" t="s">
+        <v>151</v>
+      </c>
+      <c r="E173" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="F173" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="G173" s="0" t="s">
+        <v>280</v>
+      </c>
+      <c r="H173" s="0" t="s">
+        <v>195</v>
+      </c>
+      <c r="I173" s="3">
+        <v>46315.67375</v>
+      </c>
+      <c r="J173" s="3">
+        <v>46308.3820833333</v>
+      </c>
+      <c r="K173" s="0" t="s">
+        <v>159</v>
+      </c>
+      <c r="L173" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="M173" s="3">
+        <v>46308.3820833333</v>
+      </c>
+      <c r="N173" s="3">
+        <v>46315.67375</v>
+      </c>
+      <c r="O173" s="3"/>
     </row>
   </sheetData>
   <headerFooter/>

</xml_diff>